<commit_message>
[auto-snapshot] 2026-04-15 16:00 | onda-hompage | 47 files
</commit_message>
<xml_diff>
--- a/naver-place-crawler/results_derma/강화군_피부과.xlsx
+++ b/naver-place-crawler/results_derma/강화군_피부과.xlsx
@@ -417,14 +417,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V12"/>
+  <dimension ref="A1:V25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="32" customWidth="1" min="7" max="7"/>
     <col width="47" customWidth="1" min="8" max="8"/>
@@ -559,25 +559,25 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>가정의학과</t>
+          <t>피부과</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>큰나무의원</t>
+          <t>본의원</t>
         </is>
       </c>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>032-233-7588</t>
+          <t>032-933-8765</t>
         </is>
       </c>
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
-          <t>인천광역시 강화군 강화읍 중앙로 9</t>
+          <t>인천광역시 강화군 강화읍 강화대로 395 준프라자빌딩</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -617,13 +617,13 @@
         </is>
       </c>
       <c r="P2" t="n">
-        <v>258</v>
+        <v>409</v>
       </c>
       <c r="Q2" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="R2" t="n">
-        <v>260</v>
+        <v>419</v>
       </c>
       <c r="S2" t="inlineStr">
         <is>
@@ -632,12 +632,12 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>36797044</t>
+          <t>13070802</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/36797044</t>
+          <t>https://m.place.naver.com/place/13070802</t>
         </is>
       </c>
       <c r="V2" t="inlineStr">
@@ -649,21 +649,25 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>병원,의원</t>
+          <t>가정의학과</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>정 의원</t>
+          <t>큰나무의원</t>
         </is>
       </c>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>032-233-7588</t>
+        </is>
+      </c>
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t>인천광역시 강화군 강화읍 강화대로 395</t>
+          <t>인천광역시 강화군 강화읍 중앙로 9</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -703,13 +707,13 @@
         </is>
       </c>
       <c r="P3" t="n">
+        <v>258</v>
+      </c>
+      <c r="Q3" t="n">
         <v>2</v>
       </c>
-      <c r="Q3" t="n">
-        <v>0</v>
-      </c>
       <c r="R3" t="n">
-        <v>2</v>
+        <v>260</v>
       </c>
       <c r="S3" t="inlineStr">
         <is>
@@ -718,12 +722,12 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>1704510554</t>
+          <t>36797044</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1704510554</t>
+          <t>https://m.place.naver.com/place/36797044</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
@@ -735,29 +739,29 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>외과</t>
+          <t>내과</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>인성의원</t>
+          <t>임성식내과의원</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>djawnsdn2630@naver.com</t>
+          <t>ghssghss@naver.com</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>032-932-4455</t>
+          <t>032-932-3375</t>
         </is>
       </c>
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
-          <t>인천광역시 강화군 강화읍 중앙로 23</t>
+          <t>인천광역시 강화군 강화읍 강화대로 395 3층</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -797,13 +801,13 @@
         </is>
       </c>
       <c r="P4" t="n">
-        <v>603</v>
+        <v>362</v>
       </c>
       <c r="Q4" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="R4" t="n">
-        <v>611</v>
+        <v>363</v>
       </c>
       <c r="S4" t="inlineStr">
         <is>
@@ -812,12 +816,12 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>13241435</t>
+          <t>1587926050</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/13241435</t>
+          <t>https://m.place.naver.com/place/1587926050</t>
         </is>
       </c>
       <c r="V4" t="inlineStr">
@@ -829,34 +833,26 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>한의원</t>
+          <t>병원,의원</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>늘곁한의원</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>cheolsoo58@naver.com</t>
-        </is>
-      </c>
+          <t>정 의원</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>032-716-5975</t>
-        </is>
-      </c>
+      <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
-          <t>인천광역시 강화군 강화읍 강화대로 334 1층</t>
+          <t>인천광역시 강화군 강화읍 강화대로 395</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/alwayswithyou_kmed/</t>
+          <t>X</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -866,7 +862,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -887,17 +883,17 @@
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="P5" t="n">
-        <v>82</v>
+        <v>2</v>
       </c>
       <c r="Q5" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="R5" t="n">
-        <v>85</v>
+        <v>2</v>
       </c>
       <c r="S5" t="inlineStr">
         <is>
@@ -906,12 +902,12 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>1610115216</t>
+          <t>1704510554</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1610115216</t>
+          <t>https://m.place.naver.com/place/1704510554</t>
         </is>
       </c>
       <c r="V5" t="inlineStr">
@@ -923,29 +919,29 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>한의원</t>
+          <t>병원,의원</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>우리한의원</t>
+          <t>길상의원</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>1firstdoctor@naver.com</t>
+          <t>bsing975@naver.com</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>032-932-9330</t>
+          <t>032-937-5105</t>
         </is>
       </c>
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>인천광역시 강화군 강화읍 강화대로 416</t>
+          <t>인천광역시 강화군 길상면 온수길 23 2층 길상의원</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -985,13 +981,13 @@
         </is>
       </c>
       <c r="P6" t="n">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="Q6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="R6" t="n">
-        <v>174</v>
+        <v>168</v>
       </c>
       <c r="S6" t="inlineStr">
         <is>
@@ -1000,12 +996,12 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>36332213</t>
+          <t>13241476</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/36332213</t>
+          <t>https://m.place.naver.com/place/13241476</t>
         </is>
       </c>
       <c r="V6" t="inlineStr">
@@ -1017,25 +1013,25 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>한의원</t>
+          <t>보건지소</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>성심한의원</t>
+          <t>주문보건지소</t>
         </is>
       </c>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>032-937-8122</t>
+          <t>032-932-7008</t>
         </is>
       </c>
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>인천광역시 강화군 길상면 강화동로 9</t>
+          <t>인천광역시 강화군 서도면 주문도1길 16-1</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -1075,13 +1071,13 @@
         </is>
       </c>
       <c r="P7" t="n">
-        <v>95</v>
+        <v>0</v>
       </c>
       <c r="Q7" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="R7" t="n">
-        <v>96</v>
+        <v>5</v>
       </c>
       <c r="S7" t="inlineStr">
         <is>
@@ -1090,12 +1086,12 @@
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>33586681</t>
+          <t>19522409</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/33586681</t>
+          <t>https://m.place.naver.com/place/19522409</t>
         </is>
       </c>
       <c r="V7" t="inlineStr">
@@ -1107,34 +1103,34 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>한의원</t>
+          <t>보건진료소</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>경희백향한의원</t>
+          <t>볼음보건지소</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>avalon234@naver.com</t>
+          <t>fixyourdayhere@naver.com</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>032-932-1029</t>
+          <t>032-932-7104</t>
         </is>
       </c>
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>인천광역시 강화군 강화읍 강화대로404번길 4</t>
+          <t>인천광역시 강화군 서도면 볼음도길 174</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>http://blog.daum.net/chance-4u</t>
+          <t>X</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -1144,7 +1140,7 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -1169,13 +1165,13 @@
         </is>
       </c>
       <c r="P8" t="n">
-        <v>23</v>
+        <v>0</v>
       </c>
       <c r="Q8" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="R8" t="n">
-        <v>23</v>
+        <v>6</v>
       </c>
       <c r="S8" t="inlineStr">
         <is>
@@ -1184,12 +1180,12 @@
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>19531496</t>
+          <t>19522461</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/19531496</t>
+          <t>https://m.place.naver.com/place/19522461</t>
         </is>
       </c>
       <c r="V8" t="inlineStr">
@@ -1201,34 +1197,34 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>한의원</t>
+          <t>외과</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>강화부부한의원</t>
+          <t>인성의원</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>ganghwabubu@naver.com</t>
+          <t>djawnsdn2630@naver.com</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>032-934-5533</t>
+          <t>032-932-4455</t>
         </is>
       </c>
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
-          <t>인천광역시 강화군 강화읍 향나무길 22</t>
+          <t>인천광역시 강화군 강화읍 중앙로 23</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/ganghwabubu</t>
+          <t>X</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -1238,12 +1234,12 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
@@ -1259,17 +1255,17 @@
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="P9" t="n">
-        <v>29</v>
+        <v>603</v>
       </c>
       <c r="Q9" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="R9" t="n">
-        <v>32</v>
+        <v>611</v>
       </c>
       <c r="S9" t="inlineStr">
         <is>
@@ -1278,12 +1274,12 @@
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>13241465</t>
+          <t>13241435</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/13241465</t>
+          <t>https://m.place.naver.com/place/13241435</t>
         </is>
       </c>
       <c r="V9" t="inlineStr">
@@ -1295,35 +1291,39 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>한의원</t>
+          <t>요양병원</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>제일한의원</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr"/>
+          <t>강화요양병원</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>ganghwa_hospital@naver.com</t>
+        </is>
+      </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>032-933-0087</t>
+          <t>032-937-0639</t>
         </is>
       </c>
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
-          <t>인천광역시 강화군 강화읍 남문로 75</t>
+          <t>인천광역시 강화군 길상면 강화동로 181 강화요양병원</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>https://ganghwahospital.com/</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -1353,13 +1353,13 @@
         </is>
       </c>
       <c r="P10" t="n">
-        <v>63</v>
+        <v>10</v>
       </c>
       <c r="Q10" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="R10" t="n">
-        <v>64</v>
+        <v>15</v>
       </c>
       <c r="S10" t="inlineStr">
         <is>
@@ -1368,12 +1368,12 @@
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>20713404</t>
+          <t>1937631564</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/20713404</t>
+          <t>https://m.place.naver.com/place/1937631564</t>
         </is>
       </c>
       <c r="V10" t="inlineStr">
@@ -1390,29 +1390,29 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>용정한의원</t>
+          <t>늘곁한의원</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>mintchoco_s@naver.com</t>
+          <t>cheolsoo58@naver.com</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>032-933-4048</t>
+          <t>032-716-5975</t>
         </is>
       </c>
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
-          <t>인천광역시 강화군 강화읍 갑룡길 118</t>
+          <t>인천광역시 강화군 강화읍 강화대로 334 1층</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>https://www.instagram.com/alwayswithyou_kmed/</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1422,7 +1422,7 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -1443,17 +1443,17 @@
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="P11" t="n">
-        <v>158</v>
+        <v>82</v>
       </c>
       <c r="Q11" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="R11" t="n">
-        <v>158</v>
+        <v>85</v>
       </c>
       <c r="S11" t="inlineStr">
         <is>
@@ -1462,12 +1462,12 @@
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>32473020</t>
+          <t>1610115216</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/32473020</t>
+          <t>https://m.place.naver.com/place/1610115216</t>
         </is>
       </c>
       <c r="V11" t="inlineStr">
@@ -1484,24 +1484,24 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>경희새벽한의원</t>
+          <t>우리한의원</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>bottlejean@naver.com</t>
+          <t>1firstdoctor@naver.com</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>032-932-7582</t>
+          <t>032-932-9330</t>
         </is>
       </c>
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
-          <t>인천광역시 강화군 강화읍 중앙로 23 (일석빌딩) 1층</t>
+          <t>인천광역시 강화군 강화읍 강화대로 416</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1541,30 +1541,1240 @@
         </is>
       </c>
       <c r="P12" t="n">
+        <v>170</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>4</v>
+      </c>
+      <c r="R12" t="n">
+        <v>174</v>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>36332213</t>
+        </is>
+      </c>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/36332213</t>
+        </is>
+      </c>
+      <c r="V12" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>한의원</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>성심한의원</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr"/>
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>032-937-8122</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr"/>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>인천광역시 강화군 길상면 강화동로 9</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr"/>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="P13" t="n">
+        <v>95</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>1</v>
+      </c>
+      <c r="R13" t="n">
+        <v>96</v>
+      </c>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T13" t="inlineStr">
+        <is>
+          <t>33586681</t>
+        </is>
+      </c>
+      <c r="U13" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/33586681</t>
+        </is>
+      </c>
+      <c r="V13" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>한의원</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>경희백향한의원</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>avalon234@naver.com</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr"/>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>032-932-1029</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr"/>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>인천광역시 강화군 강화읍 강화대로404번길 4</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>http://blog.daum.net/chance-4u</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr"/>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="P14" t="n">
+        <v>23</v>
+      </c>
+      <c r="Q14" t="n">
+        <v>0</v>
+      </c>
+      <c r="R14" t="n">
+        <v>23</v>
+      </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T14" t="inlineStr">
+        <is>
+          <t>19531496</t>
+        </is>
+      </c>
+      <c r="U14" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/19531496</t>
+        </is>
+      </c>
+      <c r="V14" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>한의원</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>강화부부한의원</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>ganghwabubu@naver.com</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr"/>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>032-934-5533</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr"/>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>인천광역시 강화군 강화읍 향나무길 22</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>https://blog.naver.com/ganghwabubu</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr"/>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="P15" t="n">
+        <v>29</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>3</v>
+      </c>
+      <c r="R15" t="n">
+        <v>32</v>
+      </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T15" t="inlineStr">
+        <is>
+          <t>13241465</t>
+        </is>
+      </c>
+      <c r="U15" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/13241465</t>
+        </is>
+      </c>
+      <c r="V15" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>한의원</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>제일한의원</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr"/>
+      <c r="D16" t="inlineStr"/>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>032-933-0087</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr"/>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>인천광역시 강화군 강화읍 남문로 75</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr"/>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="P16" t="n">
+        <v>63</v>
+      </c>
+      <c r="Q16" t="n">
+        <v>1</v>
+      </c>
+      <c r="R16" t="n">
         <v>64</v>
       </c>
-      <c r="Q12" t="n">
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t>20713404</t>
+        </is>
+      </c>
+      <c r="U16" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/20713404</t>
+        </is>
+      </c>
+      <c r="V16" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>한의원</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>용정한의원</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>mintchoco_s@naver.com</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr"/>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>032-933-4048</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr"/>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>인천광역시 강화군 강화읍 갑룡길 118</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr"/>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="P17" t="n">
+        <v>158</v>
+      </c>
+      <c r="Q17" t="n">
         <v>0</v>
       </c>
-      <c r="R12" t="n">
+      <c r="R17" t="n">
+        <v>158</v>
+      </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T17" t="inlineStr">
+        <is>
+          <t>32473020</t>
+        </is>
+      </c>
+      <c r="U17" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/32473020</t>
+        </is>
+      </c>
+      <c r="V17" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>한의원</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>경희새벽한의원</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>bottlejean@naver.com</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr"/>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>032-932-7582</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>인천광역시 강화군 강화읍 중앙로 23 (일석빌딩) 1층</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr"/>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="P18" t="n">
         <v>64</v>
       </c>
-      <c r="S12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="T12" t="inlineStr">
+      <c r="Q18" t="n">
+        <v>0</v>
+      </c>
+      <c r="R18" t="n">
+        <v>64</v>
+      </c>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T18" t="inlineStr">
         <is>
           <t>21062931</t>
         </is>
       </c>
-      <c r="U12" t="inlineStr">
+      <c r="U18" t="inlineStr">
         <is>
           <t>https://m.place.naver.com/place/21062931</t>
         </is>
       </c>
-      <c r="V12" t="inlineStr">
+      <c r="V18" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>한의원</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>채준환한의원</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>mrhanbit@naver.com</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr"/>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>032-937-7574</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>인천광역시 강화군 화도면 마니산로 716</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr"/>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="P19" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q19" t="n">
+        <v>1</v>
+      </c>
+      <c r="R19" t="n">
+        <v>1</v>
+      </c>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T19" t="inlineStr">
+        <is>
+          <t>1808971613</t>
+        </is>
+      </c>
+      <c r="U19" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/1808971613</t>
+        </is>
+      </c>
+      <c r="V19" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>한의원</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>더조은경희한의원</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>kkslmjlove@naver.com</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr"/>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>0507-1308-8276</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>인천광역시 강화군 강화읍 충렬사로 25 3층 303호</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>https://blog.naver.com/kkslmjlove</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr"/>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="P20" t="n">
+        <v>152</v>
+      </c>
+      <c r="Q20" t="n">
+        <v>51</v>
+      </c>
+      <c r="R20" t="n">
+        <v>203</v>
+      </c>
+      <c r="S20" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T20" t="inlineStr">
+        <is>
+          <t>1964704753</t>
+        </is>
+      </c>
+      <c r="U20" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/1964704753</t>
+        </is>
+      </c>
+      <c r="V20" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>한의원</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>명인한의원</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>brightin5234@naver.com</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr"/>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>032-934-5805</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>인천광역시 강화군 강화읍 강화대로 375</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr"/>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="P21" t="n">
+        <v>56</v>
+      </c>
+      <c r="Q21" t="n">
+        <v>0</v>
+      </c>
+      <c r="R21" t="n">
+        <v>56</v>
+      </c>
+      <c r="S21" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T21" t="inlineStr">
+        <is>
+          <t>19518812</t>
+        </is>
+      </c>
+      <c r="U21" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/19518812</t>
+        </is>
+      </c>
+      <c r="V21" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>한의원</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>감초한의원</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr"/>
+      <c r="D22" t="inlineStr"/>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>032-934-2163</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>인천광역시 강화군 강화읍 청하동길9번길 7</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr"/>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="P22" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q22" t="n">
+        <v>0</v>
+      </c>
+      <c r="R22" t="n">
+        <v>10</v>
+      </c>
+      <c r="S22" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T22" t="inlineStr">
+        <is>
+          <t>13241455</t>
+        </is>
+      </c>
+      <c r="U22" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/13241455</t>
+        </is>
+      </c>
+      <c r="V22" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>한의원</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>자성한의원</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>jasungkmd@naver.com</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr"/>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>032-719-8880</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>인천광역시 강화군 강화읍 중앙로 68 2층 자성한의원</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>https://blog.naver.com/jasungkmd</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr"/>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="P23" t="n">
+        <v>66</v>
+      </c>
+      <c r="Q23" t="n">
+        <v>7</v>
+      </c>
+      <c r="R23" t="n">
+        <v>73</v>
+      </c>
+      <c r="S23" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T23" t="inlineStr">
+        <is>
+          <t>1228477451</t>
+        </is>
+      </c>
+      <c r="U23" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/1228477451</t>
+        </is>
+      </c>
+      <c r="V23" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>한의원</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>강화한의원</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>khomsin@naver.com</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr"/>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>032-934-6336</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>인천광역시 강화군 강화읍 강화대로393번길 5</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>https://blog.naver.com/khomsin</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr"/>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="P24" t="n">
+        <v>36</v>
+      </c>
+      <c r="Q24" t="n">
+        <v>1</v>
+      </c>
+      <c r="R24" t="n">
+        <v>37</v>
+      </c>
+      <c r="S24" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T24" t="inlineStr">
+        <is>
+          <t>13241468</t>
+        </is>
+      </c>
+      <c r="U24" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/13241468</t>
+        </is>
+      </c>
+      <c r="V24" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>한의원</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>길상한의원</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>bsing975@naver.com</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr"/>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>032-937-8565</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr"/>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>인천광역시 강화군 길상면 마니산로 53</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr"/>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="P25" t="n">
+        <v>67</v>
+      </c>
+      <c r="Q25" t="n">
+        <v>0</v>
+      </c>
+      <c r="R25" t="n">
+        <v>67</v>
+      </c>
+      <c r="S25" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T25" t="inlineStr">
+        <is>
+          <t>13116068</t>
+        </is>
+      </c>
+      <c r="U25" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/13116068</t>
+        </is>
+      </c>
+      <c r="V25" t="inlineStr">
         <is>
           <t>2026-04-15</t>
         </is>

</xml_diff>